<commit_message>
Excel: planilhas verificadas no Excel e gráficos corrigidos
Categorias dos gráficos como texto, títulos sem sobreposição, eixos e
legenda visíveis. Prints trocados por capturas do Excel.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AcydA1t7SxpgmSydUbNguB
</commit_message>
<xml_diff>
--- a/projetos/excel/controle-imposto-de-renda/controle-imposto-de-renda.xlsx
+++ b/projetos/excel/controle-imposto-de-renda/controle-imposto-de-renda.xlsx
@@ -405,6 +405,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <pieChart>
@@ -418,9 +419,9 @@
             </a:ln>
           </spPr>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Resumo'!$B$10:$B$14</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -464,6 +465,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <barChart>
@@ -481,9 +483,9 @@
             </a:ln>
           </spPr>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Resumo'!$B$18:$B$22</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -500,6 +502,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
@@ -510,12 +513,25 @@
         <axId val="100"/>
         <scaling>
           <orientation val="minMax"/>
+          <min val="0"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorGridlines/>
+        <majorGridlines>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="6350">
+              <a:solidFill>
+                <a:srgbClr val="D9D9D9"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+        </majorGridlines>
+        <numFmt formatCode="#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
+        <majorUnit val="2000"/>
       </valAx>
     </plotArea>
     <plotVisOnly val="1"/>

</xml_diff>